<commit_message>
fixed istd normalization bug
</commit_message>
<xml_diff>
--- a/example1-metabolomics/results-A/pca/pca_norm_FemMHFD_over_FemMRD.xlsx
+++ b/example1-metabolomics/results-A/pca/pca_norm_FemMHFD_over_FemMRD.xlsx
@@ -494,40 +494,40 @@
         <v>13</v>
       </c>
       <c r="B2" t="n">
-        <v>0.261823987556319</v>
+        <v>0.266917598320151</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0909518690975585</v>
+        <v>0.0999188514822863</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.12888114165591</v>
+        <v>-0.140572600909419</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.204763082410285</v>
+        <v>-0.167109283988825</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.242305530105312</v>
+        <v>-0.305377741000997</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.171727750404981</v>
+        <v>-0.0469796050769309</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.0206765783749514</v>
+        <v>-0.0242665308521886</v>
       </c>
       <c r="I2" t="n">
-        <v>0.145384630996037</v>
+        <v>0.158792099341916</v>
       </c>
       <c r="J2" t="n">
-        <v>0.410043702212266</v>
+        <v>0.460100911802354</v>
       </c>
       <c r="K2" t="n">
-        <v>-0.329130066074809</v>
+        <v>-0.291513838831475</v>
       </c>
       <c r="L2" t="n">
-        <v>0.127722711689959</v>
+        <v>0.0744007162663069</v>
       </c>
       <c r="M2" t="n">
-        <v>-0.174449488967059</v>
+        <v>0.178205325899621</v>
       </c>
     </row>
     <row r="3">
@@ -535,40 +535,40 @@
         <v>14</v>
       </c>
       <c r="B3" t="n">
-        <v>0.0824213830714776</v>
+        <v>0.0727567348961308</v>
       </c>
       <c r="C3" t="n">
-        <v>0.018037221717249</v>
+        <v>0.0159134051580579</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.277772274403466</v>
+        <v>-0.267079133333895</v>
       </c>
       <c r="E3" t="n">
-        <v>0.105236658632026</v>
+        <v>0.054765284330109</v>
       </c>
       <c r="F3" t="n">
-        <v>0.230820418563494</v>
+        <v>0.20517130618056</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.124020241359648</v>
+        <v>-0.260297455535843</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.253510131267952</v>
+        <v>-0.241464223153545</v>
       </c>
       <c r="I3" t="n">
-        <v>-0.363914921394439</v>
+        <v>-0.373232612999263</v>
       </c>
       <c r="J3" t="n">
-        <v>-0.182488120018929</v>
+        <v>-0.0972311249999409</v>
       </c>
       <c r="K3" t="n">
-        <v>-0.285675744432915</v>
+        <v>-0.214735913476757</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.470282766238939</v>
+        <v>-0.503670830297279</v>
       </c>
       <c r="M3" t="n">
-        <v>-0.158371423703916</v>
+        <v>-0.207083591710656</v>
       </c>
     </row>
     <row r="4">
@@ -576,40 +576,40 @@
         <v>15</v>
       </c>
       <c r="B4" t="n">
-        <v>0.126544517666532</v>
+        <v>0.137675673286502</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.255308472719459</v>
+        <v>-0.250330483492937</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.175689050782482</v>
+        <v>-0.181886971838606</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0671003834734288</v>
+        <v>0.115519457271776</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.221594916595336</v>
+        <v>-0.207369496625016</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.0551714931054723</v>
+        <v>-0.0409153071080431</v>
       </c>
       <c r="H4" t="n">
-        <v>0.57456675081585</v>
+        <v>0.574158976911057</v>
       </c>
       <c r="I4" t="n">
-        <v>-0.0704952710755388</v>
+        <v>-0.077389391738392</v>
       </c>
       <c r="J4" t="n">
-        <v>-0.130013102199978</v>
+        <v>-0.0993924300267765</v>
       </c>
       <c r="K4" t="n">
-        <v>0.293137025571704</v>
+        <v>0.348283313792014</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.272939155535897</v>
+        <v>-0.230439504675671</v>
       </c>
       <c r="M4" t="n">
-        <v>-0.0812423568131396</v>
+        <v>-0.0466650128020233</v>
       </c>
     </row>
     <row r="5">
@@ -617,40 +617,40 @@
         <v>16</v>
       </c>
       <c r="B5" t="n">
-        <v>0.0856402864903987</v>
+        <v>0.0953560476400098</v>
       </c>
       <c r="C5" t="n">
-        <v>0.149282382294372</v>
+        <v>0.157909238108493</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.22469974311461</v>
+        <v>-0.235514272967712</v>
       </c>
       <c r="E5" t="n">
-        <v>0.289221410674635</v>
+        <v>0.408999022427288</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.432386261901745</v>
+        <v>-0.296231894403339</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1741423239906</v>
+        <v>0.146442373735303</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.385894663860757</v>
+        <v>-0.38870070365194</v>
       </c>
       <c r="I5" t="n">
-        <v>0.186177830443273</v>
+        <v>0.18131190647429</v>
       </c>
       <c r="J5" t="n">
-        <v>-0.183580234421193</v>
+        <v>-0.213580145067502</v>
       </c>
       <c r="K5" t="n">
-        <v>0.141371111823671</v>
+        <v>0.179378704060505</v>
       </c>
       <c r="L5" t="n">
-        <v>-0.290170070653929</v>
+        <v>-0.273272209448954</v>
       </c>
       <c r="M5" t="n">
-        <v>-0.00605385040295923</v>
+        <v>-0.0900791428068817</v>
       </c>
     </row>
     <row r="6">
@@ -658,40 +658,40 @@
         <v>17</v>
       </c>
       <c r="B6" t="n">
-        <v>0.204555978013453</v>
+        <v>0.193258145364631</v>
       </c>
       <c r="C6" t="n">
-        <v>0.107564409647713</v>
+        <v>0.108726518940433</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0261098285412986</v>
+        <v>0.0274212404285158</v>
       </c>
       <c r="E6" t="n">
-        <v>0.32297412063245</v>
+        <v>0.392096938212005</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.314853549840941</v>
+        <v>-0.178734230088509</v>
       </c>
       <c r="G6" t="n">
-        <v>0.245425375806718</v>
+        <v>0.335363669817416</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.0291792893514182</v>
+        <v>-0.0358132791202799</v>
       </c>
       <c r="I6" t="n">
-        <v>-0.204477292969373</v>
+        <v>-0.195801458801908</v>
       </c>
       <c r="J6" t="n">
-        <v>0.123476446858064</v>
+        <v>0.0402515733295189</v>
       </c>
       <c r="K6" t="n">
-        <v>-0.171704314447545</v>
+        <v>-0.267875192293216</v>
       </c>
       <c r="L6" t="n">
-        <v>0.359495001516574</v>
+        <v>0.339597184817753</v>
       </c>
       <c r="M6" t="n">
-        <v>0.172953319476667</v>
+        <v>-0.173694295395321</v>
       </c>
     </row>
     <row r="7">
@@ -699,40 +699,40 @@
         <v>18</v>
       </c>
       <c r="B7" t="n">
-        <v>0.164134253701586</v>
+        <v>0.163735720093735</v>
       </c>
       <c r="C7" t="n">
-        <v>-0.106217030439773</v>
+        <v>-0.10350368580669</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.152685693529854</v>
+        <v>-0.154457705172968</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.105061880035238</v>
+        <v>-0.108227761885268</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.0240937828989338</v>
+        <v>-0.0722452355934899</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.13076750406411</v>
+        <v>-0.114737194061121</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0350781482914085</v>
+        <v>0.0405857037291267</v>
       </c>
       <c r="I7" t="n">
-        <v>-0.144163396818248</v>
+        <v>-0.147525645621885</v>
       </c>
       <c r="J7" t="n">
-        <v>-0.0560917016969105</v>
+        <v>-0.0209025657393459</v>
       </c>
       <c r="K7" t="n">
-        <v>-0.245773068770662</v>
+        <v>-0.24333719134852</v>
       </c>
       <c r="L7" t="n">
-        <v>0.0089222308584499</v>
+        <v>-0.0277664114266886</v>
       </c>
       <c r="M7" t="n">
-        <v>0.283499980332</v>
+        <v>0.0560088114268941</v>
       </c>
     </row>
     <row r="8">
@@ -740,40 +740,40 @@
         <v>19</v>
       </c>
       <c r="B8" t="n">
-        <v>0.182841457293584</v>
+        <v>0.17982295461202</v>
       </c>
       <c r="C8" t="n">
-        <v>0.357867941886482</v>
+        <v>0.361580994655096</v>
       </c>
       <c r="D8" t="n">
-        <v>0.640163318250712</v>
+        <v>0.643863209724034</v>
       </c>
       <c r="E8" t="n">
-        <v>0.109967384310386</v>
+        <v>0.0923934138702546</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.169836751568261</v>
+        <v>-0.242912994196439</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.307322565261382</v>
+        <v>-0.267280174877049</v>
       </c>
       <c r="H8" t="n">
-        <v>0.0440675973608557</v>
+        <v>0.0540293266201608</v>
       </c>
       <c r="I8" t="n">
-        <v>-0.300466805446217</v>
+        <v>-0.304807909702891</v>
       </c>
       <c r="J8" t="n">
-        <v>-0.0661998714455598</v>
+        <v>0.0055488372720253</v>
       </c>
       <c r="K8" t="n">
-        <v>-0.0017965014982206</v>
+        <v>0.0376671252943478</v>
       </c>
       <c r="L8" t="n">
-        <v>-0.201747235252088</v>
+        <v>-0.195671244486511</v>
       </c>
       <c r="M8" t="n">
-        <v>0.0889515181649555</v>
+        <v>0.095690084770231</v>
       </c>
     </row>
     <row r="9">
@@ -781,40 +781,40 @@
         <v>20</v>
       </c>
       <c r="B9" t="n">
-        <v>0.201526967140976</v>
+        <v>0.202868030098328</v>
       </c>
       <c r="C9" t="n">
-        <v>0.2964377604758</v>
+        <v>0.304508224655147</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.223041741878233</v>
+        <v>-0.233311419716194</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.047830082982413</v>
+        <v>-0.000877984038067238</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.15705073993131</v>
+        <v>-0.150358560954714</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.0353866486764969</v>
+        <v>-0.04927213113337</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.193028413435194</v>
+        <v>-0.190273269126041</v>
       </c>
       <c r="I9" t="n">
-        <v>0.214449220377252</v>
+        <v>0.211752493392904</v>
       </c>
       <c r="J9" t="n">
-        <v>-0.064641039051596</v>
+        <v>-0.0469638544115505</v>
       </c>
       <c r="K9" t="n">
-        <v>-0.00938909306908295</v>
+        <v>-0.00737491846783212</v>
       </c>
       <c r="L9" t="n">
-        <v>0.0947264264175511</v>
+        <v>0.0861745573808784</v>
       </c>
       <c r="M9" t="n">
-        <v>0.0780705976600274</v>
+        <v>0.199714684407762</v>
       </c>
     </row>
     <row r="10">
@@ -822,40 +822,40 @@
         <v>21</v>
       </c>
       <c r="B10" t="n">
-        <v>0.217974691876717</v>
+        <v>0.200442343845345</v>
       </c>
       <c r="C10" t="n">
-        <v>0.189412404781994</v>
+        <v>0.18745895933197</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.0959444920825243</v>
+        <v>-0.08805144523577</v>
       </c>
       <c r="E10" t="n">
-        <v>0.0328141004409479</v>
+        <v>-0.00841966836301479</v>
       </c>
       <c r="F10" t="n">
-        <v>0.1297039908255</v>
+        <v>0.10316927915363</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.0787233862444705</v>
+        <v>-0.077859178374418</v>
       </c>
       <c r="H10" t="n">
-        <v>0.194282974238085</v>
+        <v>0.198939139092879</v>
       </c>
       <c r="I10" t="n">
-        <v>-0.0893978263929157</v>
+        <v>-0.085658731399016</v>
       </c>
       <c r="J10" t="n">
-        <v>0.136465018773484</v>
+        <v>0.162707992468642</v>
       </c>
       <c r="K10" t="n">
-        <v>-0.149734981129422</v>
+        <v>-0.160922870743445</v>
       </c>
       <c r="L10" t="n">
-        <v>0.0393879551837127</v>
+        <v>0.0277244875803556</v>
       </c>
       <c r="M10" t="n">
-        <v>-0.208772180613785</v>
+        <v>-0.532158479607622</v>
       </c>
     </row>
     <row r="11">
@@ -863,40 +863,40 @@
         <v>22</v>
       </c>
       <c r="B11" t="n">
-        <v>0.652383172291312</v>
+        <v>0.670695669836131</v>
       </c>
       <c r="C11" t="n">
-        <v>-0.0608772937913224</v>
+        <v>-0.0403769104165487</v>
       </c>
       <c r="D11" t="n">
-        <v>0.263103944412221</v>
+        <v>0.242532749592142</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.0711837661539075</v>
+        <v>-0.0462871445064869</v>
       </c>
       <c r="F11" t="n">
-        <v>0.270198800351687</v>
+        <v>0.398212618371782</v>
       </c>
       <c r="G11" t="n">
-        <v>0.466612716106524</v>
+        <v>0.315228196107169</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.0148671777041054</v>
+        <v>-0.0241114442408963</v>
       </c>
       <c r="I11" t="n">
-        <v>0.100879347578287</v>
+        <v>0.0972339638988347</v>
       </c>
       <c r="J11" t="n">
-        <v>-0.131056338756623</v>
+        <v>-0.177527425604616</v>
       </c>
       <c r="K11" t="n">
-        <v>0.165994262712678</v>
+        <v>0.170157899902771</v>
       </c>
       <c r="L11" t="n">
-        <v>0.0212921322910992</v>
+        <v>0.0333355337252661</v>
       </c>
       <c r="M11" t="n">
-        <v>-0.154869352697951</v>
+        <v>-0.0813501732351214</v>
       </c>
     </row>
     <row r="12">
@@ -904,40 +904,40 @@
         <v>23</v>
       </c>
       <c r="B12" t="n">
-        <v>0.0652506832051672</v>
+        <v>0.0806216261515852</v>
       </c>
       <c r="C12" t="n">
-        <v>0.241966226864579</v>
+        <v>0.254111229129962</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.15911641130623</v>
+        <v>-0.195105871797404</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.747369218214163</v>
+        <v>-0.652332876373141</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.246103008815395</v>
+        <v>-0.29367271091735</v>
       </c>
       <c r="G12" t="n">
-        <v>0.136106392013702</v>
+        <v>0.320400271938089</v>
       </c>
       <c r="H12" t="n">
-        <v>0.00442641884391315</v>
+        <v>-0.00725458134421546</v>
       </c>
       <c r="I12" t="n">
-        <v>-0.248079802011979</v>
+        <v>-0.249179681937125</v>
       </c>
       <c r="J12" t="n">
-        <v>-0.130094353673332</v>
+        <v>-0.235375631288838</v>
       </c>
       <c r="K12" t="n">
-        <v>0.250227204373608</v>
+        <v>0.232883212600329</v>
       </c>
       <c r="L12" t="n">
-        <v>-0.0781932320435871</v>
+        <v>-0.0473714086183672</v>
       </c>
       <c r="M12" t="n">
-        <v>0.117500525911035</v>
+        <v>-0.0125899535252839</v>
       </c>
     </row>
     <row r="13">
@@ -945,40 +945,40 @@
         <v>24</v>
       </c>
       <c r="B13" t="n">
-        <v>0.201047974561405</v>
+        <v>0.192007190282918</v>
       </c>
       <c r="C13" t="n">
-        <v>0.0623094172254693</v>
+        <v>0.0626908738784385</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.226079688992104</v>
+        <v>-0.21738949361485</v>
       </c>
       <c r="E13" t="n">
-        <v>0.190259215112339</v>
+        <v>0.153588116342635</v>
       </c>
       <c r="F13" t="n">
-        <v>0.172029701666297</v>
+        <v>0.161281175127637</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.152229420818781</v>
+        <v>-0.327304037370016</v>
       </c>
       <c r="H13" t="n">
-        <v>0.169281919686855</v>
+        <v>0.186557697974097</v>
       </c>
       <c r="I13" t="n">
-        <v>-0.0323442484888377</v>
+        <v>-0.0517921115048179</v>
       </c>
       <c r="J13" t="n">
-        <v>-0.454877338873454</v>
+        <v>-0.37704381768519</v>
       </c>
       <c r="K13" t="n">
-        <v>0.0482411436828322</v>
+        <v>-0.00653174699496865</v>
       </c>
       <c r="L13" t="n">
-        <v>0.357187396145959</v>
+        <v>0.356031459775657</v>
       </c>
       <c r="M13" t="n">
-        <v>0.364732174672381</v>
+        <v>0.419845332955111</v>
       </c>
     </row>
     <row r="14">
@@ -986,40 +986,40 @@
         <v>25</v>
       </c>
       <c r="B14" t="n">
-        <v>0.040718083341743</v>
+        <v>0.046261842141668</v>
       </c>
       <c r="C14" t="n">
-        <v>-0.243511134890014</v>
+        <v>-0.242284126955252</v>
       </c>
       <c r="D14" t="n">
-        <v>0.0668668417860245</v>
+        <v>0.0681758791843116</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.00394515531612606</v>
+        <v>0.000923179389756805</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.172001732481815</v>
+        <v>-0.225595149579678</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.187529740984052</v>
+        <v>-0.108930345513242</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.154793670860998</v>
+        <v>-0.156421043109793</v>
       </c>
       <c r="I14" t="n">
-        <v>-0.38311690407466</v>
+        <v>-0.378122250180929</v>
       </c>
       <c r="J14" t="n">
-        <v>0.117693050703563</v>
+        <v>0.142454539220186</v>
       </c>
       <c r="K14" t="n">
-        <v>0.315054947957502</v>
+        <v>0.27882044799774</v>
       </c>
       <c r="L14" t="n">
-        <v>0.31310898867611</v>
+        <v>0.360507257795442</v>
       </c>
       <c r="M14" t="n">
-        <v>-0.248983566389746</v>
+        <v>-0.1780350369194</v>
       </c>
     </row>
     <row r="15">
@@ -1027,40 +1027,40 @@
         <v>26</v>
       </c>
       <c r="B15" t="n">
-        <v>0.2022190382877</v>
+        <v>0.179807910770232</v>
       </c>
       <c r="C15" t="n">
-        <v>-0.0162114784790361</v>
+        <v>-0.0231455169358976</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.0290209691356127</v>
+        <v>-0.00919545377394566</v>
       </c>
       <c r="E15" t="n">
-        <v>0.0873736388969234</v>
+        <v>0.0100573355994579</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0524106955073529</v>
+        <v>-0.0576270521242974</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.357154274317897</v>
+        <v>-0.2888762892922</v>
       </c>
       <c r="H15" t="n">
-        <v>-0.143009223012616</v>
+        <v>-0.133575928789948</v>
       </c>
       <c r="I15" t="n">
-        <v>-0.0311061588007351</v>
+        <v>-0.0228384910273649</v>
       </c>
       <c r="J15" t="n">
-        <v>0.255269137118015</v>
+        <v>0.283776189201745</v>
       </c>
       <c r="K15" t="n">
-        <v>0.298611513439128</v>
+        <v>0.293924537092402</v>
       </c>
       <c r="L15" t="n">
-        <v>-0.159768089175844</v>
+        <v>-0.0855180711312355</v>
       </c>
       <c r="M15" t="n">
-        <v>0.415271891752649</v>
+        <v>0.187488838671225</v>
       </c>
     </row>
     <row r="16">
@@ -1068,40 +1068,40 @@
         <v>27</v>
       </c>
       <c r="B16" t="n">
-        <v>0.213839642236801</v>
+        <v>0.193670027421729</v>
       </c>
       <c r="C16" t="n">
-        <v>0.207202972308278</v>
+        <v>0.204428842021448</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.212714473043064</v>
+        <v>-0.204681681288321</v>
       </c>
       <c r="E16" t="n">
-        <v>0.0497087682391856</v>
+        <v>0.0117981169435119</v>
       </c>
       <c r="F16" t="n">
-        <v>0.176556828846553</v>
+        <v>0.179495670745444</v>
       </c>
       <c r="G16" t="n">
-        <v>0.0150207091988011</v>
+        <v>-0.00197666396867636</v>
       </c>
       <c r="H16" t="n">
-        <v>0.19425476563728</v>
+        <v>0.19707349283945</v>
       </c>
       <c r="I16" t="n">
-        <v>-0.107281193188181</v>
+        <v>-0.103374142372259</v>
       </c>
       <c r="J16" t="n">
-        <v>0.124890096373546</v>
+        <v>0.13071546314856</v>
       </c>
       <c r="K16" t="n">
-        <v>-0.0973165369330792</v>
+        <v>-0.105651583549266</v>
       </c>
       <c r="L16" t="n">
-        <v>-0.0586032156537868</v>
+        <v>-0.0592770335863605</v>
       </c>
       <c r="M16" t="n">
-        <v>-0.219682852984748</v>
+        <v>0.0811712304086318</v>
       </c>
     </row>
     <row r="17">
@@ -1109,40 +1109,40 @@
         <v>28</v>
       </c>
       <c r="B17" t="n">
-        <v>0.0401209973300996</v>
+        <v>0.0471542324338527</v>
       </c>
       <c r="C17" t="n">
-        <v>-0.293845159907592</v>
+        <v>-0.291541570014217</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.0917634332488872</v>
+        <v>-0.0963378712058916</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.168103649678258</v>
+        <v>-0.159851195665296</v>
       </c>
       <c r="F17" t="n">
-        <v>-0.0589919166160472</v>
+        <v>-0.106325022994256</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.0987792439485557</v>
+        <v>-0.0747586112526254</v>
       </c>
       <c r="H17" t="n">
-        <v>-0.0969719363733764</v>
+        <v>-0.0918961997624529</v>
       </c>
       <c r="I17" t="n">
-        <v>-0.218211160357999</v>
+        <v>-0.225855887129439</v>
       </c>
       <c r="J17" t="n">
-        <v>-0.21180933419482</v>
+        <v>-0.202565212501431</v>
       </c>
       <c r="K17" t="n">
-        <v>-0.259584792097831</v>
+        <v>-0.304044151595565</v>
       </c>
       <c r="L17" t="n">
-        <v>0.241258868754758</v>
+        <v>0.194431673363172</v>
       </c>
       <c r="M17" t="n">
-        <v>0.0465894690481641</v>
+        <v>-0.0843065443280578</v>
       </c>
     </row>
     <row r="18">
@@ -1150,40 +1150,40 @@
         <v>29</v>
       </c>
       <c r="B18" t="n">
-        <v>0.142143541485397</v>
+        <v>0.152580625724042</v>
       </c>
       <c r="C18" t="n">
-        <v>-0.347045125626102</v>
+        <v>-0.342080612185641</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.0396882434120862</v>
+        <v>-0.0425534043374853</v>
       </c>
       <c r="E18" t="n">
-        <v>0.067185828010837</v>
+        <v>0.078538979772126</v>
       </c>
       <c r="F18" t="n">
-        <v>0.0770811537319342</v>
+        <v>0.142693578047003</v>
       </c>
       <c r="G18" t="n">
-        <v>0.195849814599425</v>
+        <v>0.144853837460151</v>
       </c>
       <c r="H18" t="n">
-        <v>-0.240115456783875</v>
+        <v>-0.247358973956437</v>
       </c>
       <c r="I18" t="n">
-        <v>-0.188845592713504</v>
+        <v>-0.185247565897638</v>
       </c>
       <c r="J18" t="n">
-        <v>0.0690781829932136</v>
+        <v>0.0567508980293019</v>
       </c>
       <c r="K18" t="n">
-        <v>0.0250493531103325</v>
+        <v>0.0459048581213277</v>
       </c>
       <c r="L18" t="n">
-        <v>-0.0975689064778863</v>
+        <v>-0.0946710899432854</v>
       </c>
       <c r="M18" t="n">
-        <v>0.135525636057815</v>
+        <v>0.221440144762873</v>
       </c>
     </row>
     <row r="19">
@@ -1191,40 +1191,40 @@
         <v>30</v>
       </c>
       <c r="B19" t="n">
-        <v>0.174100753587423</v>
+        <v>0.156949087035782</v>
       </c>
       <c r="C19" t="n">
-        <v>0.03179679194328</v>
+        <v>0.0270093436066815</v>
       </c>
       <c r="D19" t="n">
-        <v>-0.0111124692343541</v>
+        <v>0.00113547044734224</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.151843797592227</v>
+        <v>-0.250769056498645</v>
       </c>
       <c r="F19" t="n">
-        <v>0.308323365358721</v>
+        <v>0.186901945081111</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.248601349991753</v>
+        <v>-0.250061400401633</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.0332610747316528</v>
+        <v>-0.0231497285842364</v>
       </c>
       <c r="I19" t="n">
-        <v>0.23798962904381</v>
+        <v>0.240593299352939</v>
       </c>
       <c r="J19" t="n">
-        <v>0.124820731039333</v>
+        <v>0.148239252790244</v>
       </c>
       <c r="K19" t="n">
-        <v>0.0346568963964091</v>
+        <v>0.0291553035810234</v>
       </c>
       <c r="L19" t="n">
-        <v>-0.0767301987798236</v>
+        <v>-0.0544693412548358</v>
       </c>
       <c r="M19" t="n">
-        <v>0.162326024162437</v>
+        <v>-0.133681902662536</v>
       </c>
     </row>
     <row r="20">
@@ -1232,40 +1232,40 @@
         <v>31</v>
       </c>
       <c r="B20" t="n">
-        <v>0.121566584328781</v>
+        <v>0.127421882694707</v>
       </c>
       <c r="C20" t="n">
-        <v>-0.32291566213173</v>
+        <v>-0.320536054832126</v>
       </c>
       <c r="D20" t="n">
-        <v>0.0211217035730356</v>
+        <v>0.016669722242292</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.0307974502394154</v>
+        <v>0.000585351010838</v>
       </c>
       <c r="F20" t="n">
-        <v>-0.144544497173199</v>
+        <v>-0.111645260573506</v>
       </c>
       <c r="G20" t="n">
-        <v>0.124743597057611</v>
+        <v>0.243514221149521</v>
       </c>
       <c r="H20" t="n">
-        <v>0.144946985645492</v>
+        <v>0.134363842045246</v>
       </c>
       <c r="I20" t="n">
-        <v>0.165977831936468</v>
+        <v>0.179280082088237</v>
       </c>
       <c r="J20" t="n">
-        <v>0.335284109762999</v>
+        <v>0.281325154867669</v>
       </c>
       <c r="K20" t="n">
-        <v>-0.111832724313801</v>
+        <v>-0.0838526017783935</v>
       </c>
       <c r="L20" t="n">
-        <v>-0.208692183910258</v>
+        <v>-0.217030846632039</v>
       </c>
       <c r="M20" t="n">
-        <v>0.367840092373898</v>
+        <v>0.0362060966769855</v>
       </c>
     </row>
     <row r="21">
@@ -1273,40 +1273,40 @@
         <v>32</v>
       </c>
       <c r="B21" t="n">
-        <v>0.12521317038752</v>
+        <v>0.124994658991987</v>
       </c>
       <c r="C21" t="n">
-        <v>-0.0880609545942742</v>
+        <v>-0.0860039686340764</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.162239601357317</v>
+        <v>-0.162449806457671</v>
       </c>
       <c r="E21" t="n">
-        <v>0.156885884136749</v>
+        <v>0.194731367156146</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.186676968239022</v>
+        <v>-0.141333159690316</v>
       </c>
       <c r="G21" t="n">
-        <v>0.0326701615236214</v>
+        <v>0.0757945592258505</v>
       </c>
       <c r="H21" t="n">
-        <v>0.183096006460325</v>
+        <v>0.178374458192286</v>
       </c>
       <c r="I21" t="n">
-        <v>-0.205927788011346</v>
+        <v>-0.199900039209401</v>
       </c>
       <c r="J21" t="n">
-        <v>0.169371480848572</v>
+        <v>0.18201815484817</v>
       </c>
       <c r="K21" t="n">
-        <v>-0.00826240540674091</v>
+        <v>0.0186635038527177</v>
       </c>
       <c r="L21" t="n">
-        <v>-0.103334224005365</v>
+        <v>-0.0998549883848211</v>
       </c>
       <c r="M21" t="n">
-        <v>-0.128765091870444</v>
+        <v>0.189080502704326</v>
       </c>
     </row>
     <row r="22">
@@ -1314,40 +1314,40 @@
         <v>33</v>
       </c>
       <c r="B22" t="n">
-        <v>0.0988946148734987</v>
+        <v>0.0810036011862554</v>
       </c>
       <c r="C22" t="n">
-        <v>0.00860687582293091</v>
+        <v>0.00226089694485064</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.174519667006554</v>
+        <v>-0.159984449594536</v>
       </c>
       <c r="E22" t="n">
-        <v>0.136087446648774</v>
+        <v>0.103742542733434</v>
       </c>
       <c r="F22" t="n">
-        <v>-0.0873535141544104</v>
+        <v>-0.157805961464106</v>
       </c>
       <c r="G22" t="n">
-        <v>-0.311912745034816</v>
+        <v>-0.276533522393201</v>
       </c>
       <c r="H22" t="n">
-        <v>0.0748289791645003</v>
+        <v>0.0881082541844405</v>
       </c>
       <c r="I22" t="n">
-        <v>0.269940258751366</v>
+        <v>0.266442880071433</v>
       </c>
       <c r="J22" t="n">
-        <v>-0.066012892210387</v>
+        <v>-0.0533413759589493</v>
       </c>
       <c r="K22" t="n">
-        <v>0.261856083489715</v>
+        <v>0.207817880478081</v>
       </c>
       <c r="L22" t="n">
-        <v>0.133367153570221</v>
+        <v>0.186864988659716</v>
       </c>
       <c r="M22" t="n">
-        <v>-0.229377979225464</v>
+        <v>-0.422425462862167</v>
       </c>
     </row>
     <row r="23">
@@ -1355,40 +1355,40 @@
         <v>34</v>
       </c>
       <c r="B23" t="n">
-        <v>0.14513446713389</v>
+        <v>0.157226685567984</v>
       </c>
       <c r="C23" t="n">
-        <v>-0.2499859784346</v>
+        <v>-0.244015012185201</v>
       </c>
       <c r="D23" t="n">
-        <v>0.258511732783937</v>
+        <v>0.250404500821674</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.107458689521634</v>
+        <v>-0.0701047186579953</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.293965423624414</v>
+        <v>-0.345683897124219</v>
       </c>
       <c r="G23" t="n">
-        <v>-0.185063701535071</v>
+        <v>-0.115877441336365</v>
       </c>
       <c r="H23" t="n">
-        <v>0.0813791302474516</v>
+        <v>0.0931621955192467</v>
       </c>
       <c r="I23" t="n">
-        <v>0.280939896060202</v>
+        <v>0.265585015129141</v>
       </c>
       <c r="J23" t="n">
-        <v>-0.39506619949702</v>
+        <v>-0.404683372846857</v>
       </c>
       <c r="K23" t="n">
-        <v>-0.36452413423452</v>
+        <v>-0.372999445248342</v>
       </c>
       <c r="L23" t="n">
-        <v>-0.117712723700194</v>
+        <v>-0.177556134165519</v>
       </c>
       <c r="M23" t="n">
-        <v>-0.102676135101231</v>
+        <v>-0.0107680961988246</v>
       </c>
     </row>
     <row r="24">
@@ -1396,40 +1396,40 @@
         <v>35</v>
       </c>
       <c r="B24" t="n">
-        <v>0.197435395037024</v>
+        <v>0.197811810162781</v>
       </c>
       <c r="C24" t="n">
-        <v>-0.279711215908623</v>
+        <v>-0.278255029734083</v>
       </c>
       <c r="D24" t="n">
-        <v>0.0416163118250918</v>
+        <v>0.0465829576843107</v>
       </c>
       <c r="E24" t="n">
-        <v>-0.0814431610208204</v>
+        <v>-0.121135974425981</v>
       </c>
       <c r="F24" t="n">
-        <v>0.0309399205245503</v>
+        <v>-0.0614018441296969</v>
       </c>
       <c r="G24" t="n">
-        <v>-0.249131858352329</v>
+        <v>-0.229869416534207</v>
       </c>
       <c r="H24" t="n">
-        <v>-0.36230942094503</v>
+        <v>-0.354490211117058</v>
       </c>
       <c r="I24" t="n">
-        <v>0.0790771536917479</v>
+        <v>0.0786132796635142</v>
       </c>
       <c r="J24" t="n">
-        <v>0.00181024263440222</v>
+        <v>0.0220334907140855</v>
       </c>
       <c r="K24" t="n">
-        <v>0.13461391740971</v>
+        <v>0.116053560340301</v>
       </c>
       <c r="L24" t="n">
-        <v>0.0514736877612704</v>
+        <v>0.0791415998759727</v>
       </c>
       <c r="M24" t="n">
-        <v>-0.233484658397465</v>
+        <v>-0.0583608580795659</v>
       </c>
     </row>
   </sheetData>

</xml_diff>